<commit_message>
init commit, started neetcode solving from stack
- Stack
- Monotonic Decreasing Stack
- Monotonic Increasing Stack
- Stack implementation (array inside)

Using Monotonic Stack we can decrease the time complexity from O(N2) to O(N)
</commit_message>
<xml_diff>
--- a/src/docs/Leetcode.xlsx
+++ b/src/docs/Leetcode.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arslan.marat\IdeaProjects\mgo\generic\Basics\src\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E3B4512-87EC-4DB2-A517-A8EEDC3897BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C95EC3-BDF0-4F19-870A-F8F068F0396A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{ED1EAF38-75F1-46AC-B64F-5B55DD06E443}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
   <si>
     <t>Topic</t>
   </si>
@@ -108,6 +108,18 @@
   </si>
   <si>
     <t>Monotonic Stack: Store indices in decreasing order of temperature. When a warmer day is found, pop() the index, calculate the day difference, and push() the current index.</t>
+  </si>
+  <si>
+    <t>853. Car Fleet</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/car-fleet/submissions/2168315498</t>
+  </si>
+  <si>
+    <t>O(NlogN)</t>
+  </si>
+  <si>
+    <t>Use the formula (target-position)/speed = time. Then create an array double [n][2] where (position, time). Sort it (time) by decrease order, then push in the stack if stack is empty or current time more than stack.peek()</t>
   </si>
 </sst>
 </file>
@@ -725,8 +737,26 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
       <c r="C6" s="5" t="s">
         <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -756,6 +786,7 @@
     <hyperlink ref="G4" r:id="rId2" xr:uid="{47D341B5-6CB4-460E-82C7-17CAC08B35C3}"/>
     <hyperlink ref="G2" r:id="rId3" xr:uid="{4BE6835D-BBCB-4C5A-B46D-070AA27739D6}"/>
     <hyperlink ref="G5" r:id="rId4" xr:uid="{9022328E-5035-43A0-844F-01868B7E442A}"/>
+    <hyperlink ref="G6" r:id="rId5" xr:uid="{3729EA78-43B6-4BDC-B177-0C2CF7A310D4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Next topic -> Two Pointers
- First Easy Task Solved
</commit_message>
<xml_diff>
--- a/src/docs/Leetcode.xlsx
+++ b/src/docs/Leetcode.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arslan.marat\IdeaProjects\mgo\generic\Basics\src\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF6A571-A3F8-40D1-92A4-728F7A1E60E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E8FC50-0913-4705-9587-8ABA3BF65D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{ED1EAF38-75F1-46AC-B64F-5B55DD06E443}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="37">
   <si>
     <t>Topic</t>
   </si>
@@ -132,6 +132,21 @@
   </si>
   <si>
     <t>2 cases -&gt; 1) if the next height is shorter, we pop this value, calculate the area (height * (i - index)) and change the start index because of 'extended back'. 2) if the next height is taller, then we just push it into the stack. Then, the values that remained in stack, we calculate the area to find max.  (height * (heights.length - index))</t>
+  </si>
+  <si>
+    <t>Two Pointers</t>
+  </si>
+  <si>
+    <t>125. Valid Palindrome</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/valid-palindrome/submissions/2170269064</t>
+  </si>
+  <si>
+    <t>O(1)</t>
+  </si>
+  <si>
+    <t>i = start, j = end, while i&lt;j iterate through the array, if the character is not digit or letter = skip, if not then compare are they the same? If not -&gt; false, if loop ends -&gt; true</t>
   </si>
 </sst>
 </file>
@@ -621,7 +636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C8EE107-1360-4CAE-8148-E378A5F6F0BB}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.5546875" customWidth="1"/>
@@ -792,6 +807,29 @@
       </c>
       <c r="G7" s="9" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -823,6 +861,7 @@
     <hyperlink ref="G5" r:id="rId4" xr:uid="{9022328E-5035-43A0-844F-01868B7E442A}"/>
     <hyperlink ref="G6" r:id="rId5" xr:uid="{3729EA78-43B6-4BDC-B177-0C2CF7A310D4}"/>
     <hyperlink ref="G7" r:id="rId6" xr:uid="{1EE6568E-6AE1-4273-8A18-CE93E51D2466}"/>
+    <hyperlink ref="G8" r:id="rId7" xr:uid="{261291C0-6966-4B64-BF7C-D8837A7834CC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Just a bit relax, returned to Arrays & Hashing topic, solve the easy one using Set
</commit_message>
<xml_diff>
--- a/src/docs/Leetcode.xlsx
+++ b/src/docs/Leetcode.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arslan.marat\IdeaProjects\mgo\generic\Basics\src\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E8FC50-0913-4705-9587-8ABA3BF65D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B60EE8-546C-441D-BC00-38C72FFD6718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{ED1EAF38-75F1-46AC-B64F-5B55DD06E443}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="41">
   <si>
     <t>Topic</t>
   </si>
@@ -147,6 +147,18 @@
   </si>
   <si>
     <t>i = start, j = end, while i&lt;j iterate through the array, if the character is not digit or letter = skip, if not then compare are they the same? If not -&gt; false, if loop ends -&gt; true</t>
+  </si>
+  <si>
+    <t>217. Contains Duplicate</t>
+  </si>
+  <si>
+    <t>Arrays &amp; Hashing</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/contains-duplicate/submissions/2171547127</t>
+  </si>
+  <si>
+    <t>Using Set and add method (returns false if duplicate value) we can iterate and add via array and if this element seen in Set (add) -&gt; return true, else return false</t>
   </si>
 </sst>
 </file>
@@ -636,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C8EE107-1360-4CAE-8148-E378A5F6F0BB}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.5546875" customWidth="1"/>
@@ -830,6 +842,29 @@
       </c>
       <c r="G8" s="9" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -862,7 +897,9 @@
     <hyperlink ref="G6" r:id="rId5" xr:uid="{3729EA78-43B6-4BDC-B177-0C2CF7A310D4}"/>
     <hyperlink ref="G7" r:id="rId6" xr:uid="{1EE6568E-6AE1-4273-8A18-CE93E51D2466}"/>
     <hyperlink ref="G8" r:id="rId7" xr:uid="{261291C0-6966-4B64-BF7C-D8837A7834CC}"/>
+    <hyperlink ref="G9" r:id="rId8" xr:uid="{4E158357-892A-4804-BF50-2D1E7BD583FD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Two Pointers topic in depth - solved 3Sum - solved Two Sum II - Input Array Is Sorted - solved Valid Palindrome
</commit_message>
<xml_diff>
--- a/src/docs/Leetcode.xlsx
+++ b/src/docs/Leetcode.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arslan.marat\IdeaProjects\mgo\generic\Basics\src\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B60EE8-546C-441D-BC00-38C72FFD6718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ACD2E0B-0A3F-4519-90B1-55853AD87704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{ED1EAF38-75F1-46AC-B64F-5B55DD06E443}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="48">
   <si>
     <t>Topic</t>
   </si>
@@ -159,6 +159,27 @@
   </si>
   <si>
     <t>Using Set and add method (returns false if duplicate value) we can iterate and add via array and if this element seen in Set (add) -&gt; return true, else return false</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/two-sum-ii-input-array-is-sorted/submissions/2178981146</t>
+  </si>
+  <si>
+    <t>167. Two Sum II - Input Array Is Sorted</t>
+  </si>
+  <si>
+    <t>Creating i as 0 and j as (n-1), if numbers[i] + numbers[j] = target &amp; i != j then return new int with positions, if numbers[i] + numbers[j] &gt; target j--, else i++</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/3sum/submissions/2179437299</t>
+  </si>
+  <si>
+    <t>15. 3Sum</t>
+  </si>
+  <si>
+    <t>O(N^2)</t>
+  </si>
+  <si>
+    <t>creating 3 pointers (i = 0, left = i + 1, right = n-1), then if sum = 0 add it to the result, then to avoid duplicates need to iterate if next or previous elements isn't the same, then at the end also move left &amp; right pointers</t>
   </si>
 </sst>
 </file>
@@ -648,7 +669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C8EE107-1360-4CAE-8148-E378A5F6F0BB}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.5546875" customWidth="1"/>
@@ -865,6 +886,52 @@
       </c>
       <c r="G9" s="9" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -898,8 +965,10 @@
     <hyperlink ref="G7" r:id="rId6" xr:uid="{1EE6568E-6AE1-4273-8A18-CE93E51D2466}"/>
     <hyperlink ref="G8" r:id="rId7" xr:uid="{261291C0-6966-4B64-BF7C-D8837A7834CC}"/>
     <hyperlink ref="G9" r:id="rId8" xr:uid="{4E158357-892A-4804-BF50-2D1E7BD583FD}"/>
+    <hyperlink ref="G10" r:id="rId9" xr:uid="{E06FA68E-9519-4480-A44E-3211E71E0222}"/>
+    <hyperlink ref="G11" r:id="rId10" xr:uid="{00CF7ED5-E858-417A-8C95-6F514DC3AAA4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TWO POINTERS TOPIC ALL SOLVED:
- ContainerWithMostWater problem solved using two pointers
- TrappingRainWater solved using three-four different approach: clean two pointers, prefix/suffix, monotonic stack

also has the variant with DP,
</commit_message>
<xml_diff>
--- a/src/docs/Leetcode.xlsx
+++ b/src/docs/Leetcode.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arslan.marat\IdeaProjects\mgo\generic\Basics\src\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ACD2E0B-0A3F-4519-90B1-55853AD87704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD64EE9E-9E08-4D5F-80C3-4CFCACA80872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{ED1EAF38-75F1-46AC-B64F-5B55DD06E443}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="58">
   <si>
     <t>Topic</t>
   </si>
@@ -180,6 +180,36 @@
   </si>
   <si>
     <t>creating 3 pointers (i = 0, left = i + 1, right = n-1), then if sum = 0 add it to the result, then to avoid duplicates need to iterate if next or previous elements isn't the same, then at the end also move left &amp; right pointers</t>
+  </si>
+  <si>
+    <t>11. Container With Most Water</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/container-with-most-water/submissions/2179690848</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Using formua -&gt; height * (right - left). If height[left] &lt; height[right] then use fomula where height is height[left] then moving left pointer, do the same if height[right] &lt; height[left]</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/trapping-rain-water/submissions/2181197762</t>
+  </si>
+  <si>
+    <t>42. Trapping Rain Water</t>
+  </si>
+  <si>
+    <t>Using formula -&gt; min(maxLeft, maxRight) - height[i], if the result is negative we take it as 0, then sum the results together, if height[left] &lt; height[right] then calculate and move pointer</t>
+  </si>
+  <si>
+    <t>Different approach using prefix/suffix method also using the formula, initialize additional two arrays maxLeft &amp; maxRight then do the same calculations</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/trapping-rain-water/submissions/2181248016</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/trapping-rain-water/submissions/2181262535</t>
+  </si>
+  <si>
+    <t>Monotonic Stack: while if stack is not empty &amp; height[i] &gt; height[stack.peek] then take and pop the val as bottomIndex, then check if stack is also not empty (not the border) continue, else break, then peek the index as leftIndex, using formula of sum += distance * boundedHeight we calc the distance as current (i) - leftIndex - 1, boundedHeight is = minimum of (height[current] and height[leftIndex]) to be sure that the water won't leak out, then-&gt;  - height[bottomIndex]. In stack we need to keep the indexes, not value</t>
   </si>
 </sst>
 </file>
@@ -669,7 +699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C8EE107-1360-4CAE-8148-E378A5F6F0BB}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.5546875" customWidth="1"/>
@@ -932,6 +962,98 @@
       </c>
       <c r="G11" s="9" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -967,8 +1089,12 @@
     <hyperlink ref="G9" r:id="rId8" xr:uid="{4E158357-892A-4804-BF50-2D1E7BD583FD}"/>
     <hyperlink ref="G10" r:id="rId9" xr:uid="{E06FA68E-9519-4480-A44E-3211E71E0222}"/>
     <hyperlink ref="G11" r:id="rId10" xr:uid="{00CF7ED5-E858-417A-8C95-6F514DC3AAA4}"/>
+    <hyperlink ref="G12" r:id="rId11" xr:uid="{4FED2025-5F0A-4A90-A4EE-48F5F0FA8175}"/>
+    <hyperlink ref="G13" r:id="rId12" xr:uid="{B1DFACDC-407D-41A4-99FC-913EBE4A0E3E}"/>
+    <hyperlink ref="G14" r:id="rId13" xr:uid="{ACCDC692-1308-4DD6-8866-08A9B2FB57C6}"/>
+    <hyperlink ref="G15" r:id="rId14" xr:uid="{7D053BB2-D56D-4E46-B3CE-ABBE5E016A39}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Arrays & Hashing topic:
- Contains Duplicate solved
- Valid Anagrams solved
- Two Sum solved
</commit_message>
<xml_diff>
--- a/src/docs/Leetcode.xlsx
+++ b/src/docs/Leetcode.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arslan.marat\IdeaProjects\mgo\generic\Basics\src\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD64EE9E-9E08-4D5F-80C3-4CFCACA80872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{040A7DED-55D1-4348-AE22-7DD07D9D811D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{ED1EAF38-75F1-46AC-B64F-5B55DD06E443}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="61">
   <si>
     <t>Topic</t>
   </si>
@@ -210,6 +210,15 @@
   </si>
   <si>
     <t>Monotonic Stack: while if stack is not empty &amp; height[i] &gt; height[stack.peek] then take and pop the val as bottomIndex, then check if stack is also not empty (not the border) continue, else break, then peek the index as leftIndex, using formula of sum += distance * boundedHeight we calc the distance as current (i) - leftIndex - 1, boundedHeight is = minimum of (height[current] and height[leftIndex]) to be sure that the water won't leak out, then-&gt;  - height[bottomIndex]. In stack we need to keep the indexes, not value</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/two-sum/submissions/2181329925</t>
+  </si>
+  <si>
+    <t>1. Two Sum</t>
+  </si>
+  <si>
+    <t>Using HashMap, go with loop we find complement = target - nums[i], if the complement exists in our map - return results, else put this value inside map</t>
   </si>
 </sst>
 </file>
@@ -699,7 +708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C8EE107-1360-4CAE-8148-E378A5F6F0BB}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.5546875" customWidth="1"/>
@@ -1054,6 +1063,29 @@
       </c>
       <c r="G15" s="9" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1093,8 +1125,9 @@
     <hyperlink ref="G13" r:id="rId12" xr:uid="{B1DFACDC-407D-41A4-99FC-913EBE4A0E3E}"/>
     <hyperlink ref="G14" r:id="rId13" xr:uid="{ACCDC692-1308-4DD6-8866-08A9B2FB57C6}"/>
     <hyperlink ref="G15" r:id="rId14" xr:uid="{7D053BB2-D56D-4E46-B3CE-ABBE5E016A39}"/>
+    <hyperlink ref="G16" r:id="rId15" xr:uid="{8F7219BE-7F2E-4C4C-B8F5-A11DD1B6F773}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>